<commit_message>
docs(tile): refresh validated TEPL profiles
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support_v03.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support_v03.xlsx
@@ -157,7 +157,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>pto-spec HEAD@a7f9aabe5e0d12fefef51f59ebc68e99873e2d47</t>
+          <t>pto-spec a7f9aabe5e0d12fefef51f59ebc68e99873e2d47@a7f9aabe5e0d12fefef51f59ebc68e99873e2d47</t>
         </is>
       </c>
     </row>
@@ -240,17 +240,17 @@
         <v>470</v>
       </c>
       <c r="C8" s="3">
-        <v>33</v>
+        <v>179</v>
       </c>
       <c r="D8" s="4">
-        <v>412</v>
+        <v>266</v>
       </c>
       <c r="E8" s="5">
         <v>25</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>38.1%</t>
         </is>
       </c>
     </row>
@@ -312,17 +312,17 @@
         <v>514</v>
       </c>
       <c r="C11" s="3">
-        <v>36</v>
+        <v>182</v>
       </c>
       <c r="D11" s="4">
-        <v>445</v>
+        <v>299</v>
       </c>
       <c r="E11" s="5">
         <v>33</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>35.4%</t>
         </is>
       </c>
     </row>
@@ -849,49 +849,49 @@
           <t>element-wise</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="AS3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -1077,49 +1077,49 @@
           <t>tile-scalar</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="AS4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -1305,34 +1305,34 @@
           <t>element-wise</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="AS5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -1533,34 +1533,34 @@
           <t>tile-scalar</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="AS6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="AS7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="AS8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -2430,7 +2430,7 @@
       </c>
       <c r="AS9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -6744,7 +6744,7 @@
       </c>
       <c r="AS28" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -7141,9 +7141,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="AH30" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="AH30" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AI30" s="6" t="inlineStr">
@@ -7193,13 +7193,13 @@
       </c>
       <c r="AR30" s="7" t="inlineStr">
         <is>
-          <t>v5_tepl_expands_profiles
-Current canonical selector 0x03B; independent raw-byte golden.</t>
+          <t>v03_tepl_expands_profiles
+Current canonical selector 0x03B; all nine defined dtypes; independent raw-byte golden.</t>
         </is>
       </c>
       <c r="AS30" s="7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -9034,39 +9034,39 @@
           <t>element-wise</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J39" s="6" t="inlineStr">
@@ -9074,9 +9074,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="K39" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr">
@@ -9247,7 +9247,7 @@
       </c>
       <c r="AS39" s="7" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -9262,49 +9262,49 @@
           <t>tile-scalar</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="K40" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr">
@@ -9475,7 +9475,7 @@
       </c>
       <c r="AS40" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -9490,39 +9490,39 @@
           <t>element-wise</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
@@ -9530,9 +9530,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="K41" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr">
@@ -9703,7 +9703,7 @@
       </c>
       <c r="AS41" s="7" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -9718,49 +9718,49 @@
           <t>tile-scalar</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L42" s="6" t="inlineStr">
@@ -9931,7 +9931,7 @@
       </c>
       <c r="AS42" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -10184,29 +10184,29 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
@@ -10214,9 +10214,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="K44" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L44" s="6" t="inlineStr">
@@ -10387,7 +10387,7 @@
       </c>
       <c r="AS44" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -10402,49 +10402,49 @@
           <t>tile-scalar</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="K45" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L45" s="6" t="inlineStr">
@@ -10615,7 +10615,7 @@
       </c>
       <c r="AS45" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -10858,34 +10858,34 @@
           <t>element-wise</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
@@ -11071,7 +11071,7 @@
       </c>
       <c r="AS47" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -11086,34 +11086,34 @@
           <t>element-wise</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
@@ -11299,7 +11299,7 @@
       </c>
       <c r="AS48" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -11314,34 +11314,34 @@
           <t>tile-scalar</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
@@ -11527,7 +11527,7 @@
       </c>
       <c r="AS49" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -17432,7 +17432,7 @@
       </c>
       <c r="AS75" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -17660,7 +17660,7 @@
       </c>
       <c r="AS76" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -17675,34 +17675,34 @@
           <t>element-wise</t>
         </is>
       </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H77" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
@@ -17888,7 +17888,7 @@
       </c>
       <c r="AS77" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -17903,34 +17903,34 @@
           <t>tile-scalar</t>
         </is>
       </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D78" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E78" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F78" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G78" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H78" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr">
@@ -18116,7 +18116,7 @@
       </c>
       <c r="AS78" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -18131,34 +18131,34 @@
           <t>element-wise</t>
         </is>
       </c>
-      <c r="C79" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D79" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="AS79" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -18359,34 +18359,34 @@
           <t>tile-scalar</t>
         </is>
       </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D80" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E80" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F80" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G80" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H80" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
@@ -18572,7 +18572,7 @@
       </c>
       <c r="AS80" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -19041,39 +19041,39 @@
           <t>element-wise</t>
         </is>
       </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="I83" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J83" s="6" t="inlineStr">
@@ -19081,9 +19081,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="K83" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="K83" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L83" s="6" t="inlineStr">
@@ -19254,7 +19254,7 @@
       </c>
       <c r="AS83" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -19279,9 +19279,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E84" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F84" s="6" t="inlineStr">
@@ -19289,9 +19289,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G84" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H84" s="6" t="inlineStr">
@@ -19299,9 +19299,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I84" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J84" s="6" t="inlineStr">
@@ -19309,9 +19309,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="K84" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L84" s="6" t="inlineStr">
@@ -19482,7 +19482,7 @@
       </c>
       <c r="AS84" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -19937,7 +19937,7 @@
       </c>
       <c r="AS86" s="7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -19952,34 +19952,34 @@
           <t>element-wise</t>
         </is>
       </c>
-      <c r="C87" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D87" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E87" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F87" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G87" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H87" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I87" s="6" t="inlineStr">
@@ -20165,7 +20165,7 @@
       </c>
       <c r="AS87" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -20180,34 +20180,34 @@
           <t>tile-scalar</t>
         </is>
       </c>
-      <c r="C88" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="D88" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="E88" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="F88" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="G88" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="H88" s="4" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I88" s="6" t="inlineStr">
@@ -20393,7 +20393,7 @@
       </c>
       <c r="AS88" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(tile): enforce PE-local cooperative matrix semantics
</commit_message>
<xml_diff>
--- a/docs/linxisa/qemu_tile_profile_support_v03.xlsx
+++ b/docs/linxisa/qemu_tile_profile_support_v03.xlsx
@@ -20749,7 +20749,7 @@
       <c r="G8" s="7" t="inlineStr">
         <is>
           <t>v03_group_mma_m16_n32_k16; v03_group_mma_m8_n16_k32
-Current ISA v0.3 PE-local operands; same ELF and independent FP32 matmul golden.</t>
+Current ISA v0.3 PE-local operands; SharedTSize class 5 means 2 KiB per PE and 8 KiB aggregate; same ELF and independent FP32 matmul golden.</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -20792,7 +20792,7 @@
       <c r="G9" s="7" t="inlineStr">
         <is>
           <t>v03_group_mma_kchunks3_m16_n32_k16
-Three K chunks prove initial TMATMUL plus repeated TMATMUL_ACC accumulation.</t>
+Three K chunks prove initial TMATMUL plus repeated explicit-C/D TMATMUL_ACC; every chunk uses SharedTSize class 5, 2 KiB per PE and 8 KiB aggregate.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -21087,7 +21087,7 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Shared S8; PE0 producer; 16x32 NORM; size class 1</t>
+          <t>Shared S8; PE0 issuer; 16x32 NORM; PE-local 512B class 3; Core4 aggregate 2KiB</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
@@ -22017,13 +22017,13 @@
       </c>
       <c r="X8" s="7" t="inlineStr">
         <is>
-          <t>v5_tile_smoke; v5_group_mma_smoke
-Generic TLSU profile remains yellow; only explicit profiles are green.</t>
+          <t>Static Shared TLOAD implementation audit
+The legacy class-1 carrier is invalid under the PE-local TSize table; class 3 execution needs a current-encoding independent-golden rerun.</t>
         </is>
       </c>
       <c r="Y8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>

</xml_diff>